<commit_message>
Only fill in Mathew's tracker scores; leave others blank pending real input
</commit_message>
<xml_diff>
--- a/Performance_Tracker.xlsx
+++ b/Performance_Tracker.xlsx
@@ -55,7 +55,7 @@
     <t xml:space="preserve">Scores: 0–100 contribution/performance score per activity, entered by the team leader based on actual team knowledge (not derived from git commit history — see note).</t>
   </si>
   <si>
-    <t xml:space="preserve">Milestone 1 (Sep 12) reflects the roster active at submission time via current member names; Kamaria Noble scored 75 for reported non-submission of deliverable work while remaining active in team communication.</t>
+    <t xml:space="preserve">Only Mathew Budnik's scores are filled in so far; other team members' cells are intentionally left blank pending real input on their contributions.</t>
   </si>
 </sst>
 </file>
@@ -586,7 +586,7 @@
         <v>100</v>
       </c>
       <c r="D2" s="5" t="n">
-        <f aca="false">AVERAGE(B2:C2)</f>
+        <f aca="false">IFERROR(AVERAGE(B2:C2),"")</f>
         <v>100</v>
       </c>
     </row>
@@ -594,60 +594,44 @@
       <c r="A3" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="7" t="n">
-        <v>75</v>
-      </c>
-      <c r="C3" s="7" t="n">
-        <v>100</v>
-      </c>
-      <c r="D3" s="8" t="n">
-        <f aca="false">AVERAGE(B3:C3)</f>
-        <v>87.5</v>
+      <c r="B3" s="7"/>
+      <c r="C3" s="7"/>
+      <c r="D3" s="8" t="str">
+        <f aca="false">IFERROR(AVERAGE(B3:C3),"")</f>
+        <v/>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="4" t="n">
-        <v>100</v>
-      </c>
-      <c r="C4" s="4" t="n">
-        <v>100</v>
-      </c>
-      <c r="D4" s="5" t="n">
-        <f aca="false">AVERAGE(B4:C4)</f>
-        <v>100</v>
+      <c r="B4" s="4"/>
+      <c r="C4" s="4"/>
+      <c r="D4" s="5" t="str">
+        <f aca="false">IFERROR(AVERAGE(B4:C4),"")</f>
+        <v/>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="7" t="n">
-        <v>100</v>
-      </c>
-      <c r="C5" s="7" t="n">
-        <v>100</v>
-      </c>
-      <c r="D5" s="8" t="n">
-        <f aca="false">AVERAGE(B5:C5)</f>
-        <v>100</v>
+      <c r="B5" s="7"/>
+      <c r="C5" s="7"/>
+      <c r="D5" s="8" t="str">
+        <f aca="false">IFERROR(AVERAGE(B5:C5),"")</f>
+        <v/>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="4" t="n">
-        <v>100</v>
-      </c>
-      <c r="C6" s="4" t="n">
-        <v>100</v>
-      </c>
-      <c r="D6" s="5" t="n">
-        <f aca="false">AVERAGE(B6:C6)</f>
-        <v>100</v>
+      <c r="B6" s="4"/>
+      <c r="C6" s="4"/>
+      <c r="D6" s="5" t="str">
+        <f aca="false">IFERROR(AVERAGE(B6:C6),"")</f>
+        <v/>
       </c>
     </row>
     <row r="9" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Score Sebastian 100 for Milestone 1 based on reviewed business rules/main transaction docs
</commit_message>
<xml_diff>
--- a/Performance_Tracker.xlsx
+++ b/Performance_Tracker.xlsx
@@ -55,7 +55,7 @@
     <t xml:space="preserve">Scores: 0–100 contribution/performance score per activity, entered by the team leader based on actual team knowledge (not derived from git commit history — see note).</t>
   </si>
   <si>
-    <t xml:space="preserve">Only Mathew Budnik's scores are filled in so far; other team members' cells are intentionally left blank pending real input on their contributions.</t>
+    <t xml:space="preserve">Mathew Budnik and Sebastian Tamayo (Milestone 1 business rules/main transaction docs, reviewed) are filled in; remaining cells are intentionally left blank pending real input on those contributions.</t>
   </si>
 </sst>
 </file>
@@ -605,11 +605,13 @@
       <c r="A4" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="4"/>
+      <c r="B4" s="4" t="n">
+        <v>100</v>
+      </c>
       <c r="C4" s="4"/>
-      <c r="D4" s="5" t="str">
+      <c r="D4" s="5" t="n">
         <f aca="false">IFERROR(AVERAGE(B4:C4),"")</f>
-        <v/>
+        <v>100</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>